<commit_message>
Clean up  from raw SQLite to SQLAlchemy,
</commit_message>
<xml_diff>
--- a/reports/school_1_report.xlsx
+++ b/reports/school_1_report.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="353" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="360" uniqueCount="38">
   <si>
     <t>Teacher</t>
   </si>
@@ -70,6 +70,9 @@
     <t>QUIZ2</t>
   </si>
   <si>
+    <t>QuizTest5</t>
+  </si>
+  <si>
     <t>ShortQ1</t>
   </si>
   <si>
@@ -91,6 +94,9 @@
     <t>abha</t>
   </si>
   <si>
+    <t>rishu</t>
+  </si>
+  <si>
     <t>aha</t>
   </si>
   <si>
@@ -106,6 +112,9 @@
     <t>wew</t>
   </si>
   <si>
+    <t>3</t>
+  </si>
+  <si>
     <t>40</t>
   </si>
   <si>
@@ -113,6 +122,9 @@
   </si>
   <si>
     <t>30</t>
+  </si>
+  <si>
+    <t>50</t>
   </si>
   <si>
     <t>9318306080</t>
@@ -481,7 +493,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M56"/>
+  <dimension ref="A1:M57"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -495,7 +507,7 @@
     <col min="9" max="9" width="13.7109375" customWidth="1"/>
     <col min="10" max="10" width="20.7109375" customWidth="1"/>
     <col min="11" max="11" width="12.7109375" customWidth="1"/>
-    <col min="12" max="13" width="21.7109375" customWidth="1"/>
+    <col min="12" max="13" width="28.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:13">
@@ -547,16 +559,16 @@
         <v>15</v>
       </c>
       <c r="C2" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="D2" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="F2" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="G2" t="s">
-        <v>33</v>
+        <v>37</v>
       </c>
       <c r="H2">
         <v>4</v>
@@ -585,7 +597,13 @@
         <v>16</v>
       </c>
       <c r="G3" t="s">
-        <v>33</v>
+        <v>37</v>
+      </c>
+      <c r="L3" s="2">
+        <v>46103.51736057608</v>
+      </c>
+      <c r="M3" s="2">
+        <v>46103.51736057608</v>
       </c>
     </row>
     <row r="4" spans="1:13">
@@ -596,16 +614,16 @@
         <v>17</v>
       </c>
       <c r="C4" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="D4" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="F4" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="G4" t="s">
-        <v>33</v>
+        <v>37</v>
       </c>
       <c r="K4">
         <v>2</v>
@@ -613,6 +631,9 @@
       <c r="L4" s="2">
         <v>46087.41199074074</v>
       </c>
+      <c r="M4" s="2">
+        <v>46103.51736057608</v>
+      </c>
     </row>
     <row r="5" spans="1:13">
       <c r="A5" t="s">
@@ -622,16 +643,16 @@
         <v>17</v>
       </c>
       <c r="C5" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="D5" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="F5" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="G5" t="s">
-        <v>33</v>
+        <v>37</v>
       </c>
       <c r="H5">
         <v>5</v>
@@ -660,16 +681,16 @@
         <v>17</v>
       </c>
       <c r="C6" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="D6" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="F6" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="G6" t="s">
-        <v>33</v>
+        <v>37</v>
       </c>
       <c r="H6">
         <v>5</v>
@@ -698,16 +719,16 @@
         <v>17</v>
       </c>
       <c r="C7" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="D7" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="F7" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="G7" t="s">
-        <v>33</v>
+        <v>37</v>
       </c>
       <c r="H7">
         <v>0</v>
@@ -736,16 +757,16 @@
         <v>17</v>
       </c>
       <c r="C8" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="D8" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="F8" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="G8" t="s">
-        <v>33</v>
+        <v>37</v>
       </c>
       <c r="H8">
         <v>0</v>
@@ -774,16 +795,16 @@
         <v>17</v>
       </c>
       <c r="C9" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="D9" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="F9" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="G9" t="s">
-        <v>33</v>
+        <v>37</v>
       </c>
       <c r="H9">
         <v>0</v>
@@ -812,16 +833,16 @@
         <v>17</v>
       </c>
       <c r="C10" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="D10" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="F10" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="G10" t="s">
-        <v>33</v>
+        <v>37</v>
       </c>
       <c r="K10">
         <v>1</v>
@@ -829,6 +850,9 @@
       <c r="L10" s="2">
         <v>46087.40681712963</v>
       </c>
+      <c r="M10" s="2">
+        <v>46103.51736057608</v>
+      </c>
     </row>
     <row r="11" spans="1:13">
       <c r="A11" t="s">
@@ -838,16 +862,16 @@
         <v>17</v>
       </c>
       <c r="C11" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="D11" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="F11" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="G11" t="s">
-        <v>33</v>
+        <v>37</v>
       </c>
       <c r="K11">
         <v>9</v>
@@ -855,6 +879,9 @@
       <c r="L11" s="2">
         <v>46087.80561342592</v>
       </c>
+      <c r="M11" s="2">
+        <v>46103.51736057608</v>
+      </c>
     </row>
     <row r="12" spans="1:13">
       <c r="A12" t="s">
@@ -864,16 +891,16 @@
         <v>17</v>
       </c>
       <c r="C12" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="D12" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="F12" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="G12" t="s">
-        <v>33</v>
+        <v>37</v>
       </c>
       <c r="H12">
         <v>0</v>
@@ -902,34 +929,37 @@
         <v>18</v>
       </c>
       <c r="C13" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="D13" t="s">
-        <v>28</v>
+        <v>26</v>
+      </c>
+      <c r="E13" t="s">
+        <v>32</v>
       </c>
       <c r="F13" t="s">
-        <v>31</v>
+        <v>36</v>
       </c>
       <c r="G13" t="s">
-        <v>33</v>
+        <v>37</v>
       </c>
       <c r="H13">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="I13">
         <v>7</v>
       </c>
       <c r="J13">
-        <v>0</v>
+        <v>28.57142857142857</v>
       </c>
       <c r="K13">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L13" s="2">
-        <v>46088.25815972222</v>
+        <v>46103.44877828533</v>
       </c>
       <c r="M13" s="2">
-        <v>46088.26086805556</v>
+        <v>46103.45007326682</v>
       </c>
     </row>
     <row r="14" spans="1:13">
@@ -937,37 +967,37 @@
         <v>14</v>
       </c>
       <c r="B14" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C14" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D14" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="F14" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="G14" t="s">
-        <v>33</v>
+        <v>37</v>
       </c>
       <c r="H14">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I14">
         <v>7</v>
       </c>
       <c r="J14">
-        <v>14.28571428571428</v>
+        <v>0</v>
       </c>
       <c r="K14">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="L14" s="2">
-        <v>46088.26832175926</v>
+        <v>46088.25815972222</v>
       </c>
       <c r="M14" s="2">
-        <v>46088.26900462963</v>
+        <v>46088.26086805556</v>
       </c>
     </row>
     <row r="15" spans="1:13">
@@ -975,37 +1005,37 @@
         <v>14</v>
       </c>
       <c r="B15" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C15" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="D15" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="F15" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="G15" t="s">
-        <v>33</v>
+        <v>37</v>
       </c>
       <c r="H15">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I15">
         <v>7</v>
       </c>
       <c r="J15">
-        <v>0</v>
+        <v>14.28571428571428</v>
       </c>
       <c r="K15">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="L15" s="2">
-        <v>46088.27410879629</v>
+        <v>46088.26832175926</v>
       </c>
       <c r="M15" s="2">
-        <v>46088.27479166666</v>
+        <v>46088.26900462963</v>
       </c>
     </row>
     <row r="16" spans="1:13">
@@ -1013,19 +1043,19 @@
         <v>14</v>
       </c>
       <c r="B16" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C16" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="D16" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="F16" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="G16" t="s">
-        <v>33</v>
+        <v>37</v>
       </c>
       <c r="H16">
         <v>0</v>
@@ -1037,13 +1067,13 @@
         <v>0</v>
       </c>
       <c r="K16">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="L16" s="2">
-        <v>46088.30446759259</v>
+        <v>46088.27410879629</v>
       </c>
       <c r="M16" s="2">
-        <v>46088.30515046296</v>
+        <v>46088.27479166666</v>
       </c>
     </row>
     <row r="17" spans="1:13">
@@ -1051,19 +1081,19 @@
         <v>14</v>
       </c>
       <c r="B17" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C17" t="s">
         <v>23</v>
       </c>
       <c r="D17" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="F17" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="G17" t="s">
-        <v>33</v>
+        <v>37</v>
       </c>
       <c r="H17">
         <v>0</v>
@@ -1075,13 +1105,13 @@
         <v>0</v>
       </c>
       <c r="K17">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="L17" s="2">
-        <v>46088.75375</v>
+        <v>46088.30446759259</v>
       </c>
       <c r="M17" s="2">
-        <v>46088.75619212963</v>
+        <v>46088.30515046296</v>
       </c>
     </row>
     <row r="18" spans="1:13">
@@ -1089,19 +1119,19 @@
         <v>14</v>
       </c>
       <c r="B18" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C18" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="D18" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="F18" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="G18" t="s">
-        <v>33</v>
+        <v>37</v>
       </c>
       <c r="H18">
         <v>0</v>
@@ -1113,13 +1143,13 @@
         <v>0</v>
       </c>
       <c r="K18">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="L18" s="2">
-        <v>46088.75642361111</v>
+        <v>46088.75375</v>
       </c>
       <c r="M18" s="2">
-        <v>46088.75710648148</v>
+        <v>46088.75619212963</v>
       </c>
     </row>
     <row r="19" spans="1:13">
@@ -1127,19 +1157,19 @@
         <v>14</v>
       </c>
       <c r="B19" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C19" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="D19" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="F19" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="G19" t="s">
-        <v>33</v>
+        <v>37</v>
       </c>
       <c r="H19">
         <v>0</v>
@@ -1151,13 +1181,13 @@
         <v>0</v>
       </c>
       <c r="K19">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="L19" s="2">
-        <v>46088.26099537037</v>
+        <v>46088.75642361111</v>
       </c>
       <c r="M19" s="2">
-        <v>46088.26809027778</v>
+        <v>46088.75710648148</v>
       </c>
     </row>
     <row r="20" spans="1:13">
@@ -1165,19 +1195,19 @@
         <v>14</v>
       </c>
       <c r="B20" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C20" t="s">
         <v>24</v>
       </c>
       <c r="D20" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="F20" t="s">
-        <v>30</v>
+        <v>35</v>
       </c>
       <c r="G20" t="s">
-        <v>33</v>
+        <v>37</v>
       </c>
       <c r="H20">
         <v>0</v>
@@ -1189,13 +1219,13 @@
         <v>0</v>
       </c>
       <c r="K20">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="L20" s="2">
-        <v>46088.25466435185</v>
+        <v>46088.26099537037</v>
       </c>
       <c r="M20" s="2">
-        <v>46088.25792824074</v>
+        <v>46088.26809027778</v>
       </c>
     </row>
     <row r="21" spans="1:13">
@@ -1203,19 +1233,19 @@
         <v>14</v>
       </c>
       <c r="B21" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C21" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="D21" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="F21" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="G21" t="s">
-        <v>33</v>
+        <v>37</v>
       </c>
       <c r="H21">
         <v>0</v>
@@ -1227,13 +1257,13 @@
         <v>0</v>
       </c>
       <c r="K21">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="L21" s="2">
-        <v>46088.74609953703</v>
+        <v>46088.25466435185</v>
       </c>
       <c r="M21" s="2">
-        <v>46088.74945601852</v>
+        <v>46088.25792824074</v>
       </c>
     </row>
     <row r="22" spans="1:13">
@@ -1241,19 +1271,19 @@
         <v>14</v>
       </c>
       <c r="B22" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C22" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="D22" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="F22" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="G22" t="s">
-        <v>33</v>
+        <v>37</v>
       </c>
       <c r="H22">
         <v>0</v>
@@ -1265,13 +1295,13 @@
         <v>0</v>
       </c>
       <c r="K22">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="L22" s="2">
-        <v>46088.74978009259</v>
+        <v>46088.74609953703</v>
       </c>
       <c r="M22" s="2">
-        <v>46088.75325231482</v>
+        <v>46088.74945601852</v>
       </c>
     </row>
     <row r="23" spans="1:13">
@@ -1282,34 +1312,34 @@
         <v>19</v>
       </c>
       <c r="C23" t="s">
-        <v>22</v>
+        <v>27</v>
       </c>
       <c r="D23" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="F23" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="G23" t="s">
-        <v>33</v>
+        <v>37</v>
       </c>
       <c r="H23">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="I23">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="J23">
-        <v>66.66666666666666</v>
+        <v>0</v>
       </c>
       <c r="K23">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="L23" s="2">
-        <v>46087.80914351852</v>
+        <v>46088.74978009259</v>
       </c>
       <c r="M23" s="2">
-        <v>46087.81076388889</v>
+        <v>46088.75325231482</v>
       </c>
     </row>
     <row r="24" spans="1:13">
@@ -1317,25 +1347,37 @@
         <v>14</v>
       </c>
       <c r="B24" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C24" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="D24" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="F24" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="G24" t="s">
-        <v>33</v>
+        <v>37</v>
+      </c>
+      <c r="H24">
+        <v>4</v>
+      </c>
+      <c r="I24">
+        <v>6</v>
+      </c>
+      <c r="J24">
+        <v>66.66666666666666</v>
       </c>
       <c r="K24">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="L24" s="2">
-        <v>46087.81924768518</v>
+        <v>46087.80914351852</v>
+      </c>
+      <c r="M24" s="2">
+        <v>46087.81076388889</v>
       </c>
     </row>
     <row r="25" spans="1:13">
@@ -1343,37 +1385,28 @@
         <v>14</v>
       </c>
       <c r="B25" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C25" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="D25" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="F25" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="G25" t="s">
-        <v>33</v>
-      </c>
-      <c r="H25">
-        <v>0</v>
-      </c>
-      <c r="I25">
-        <v>1</v>
-      </c>
-      <c r="J25">
-        <v>0</v>
+        <v>37</v>
       </c>
       <c r="K25">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L25" s="2">
-        <v>46087.81978009259</v>
+        <v>46087.81924768518</v>
       </c>
       <c r="M25" s="2">
-        <v>46087.81979166667</v>
+        <v>46103.51736058765</v>
       </c>
     </row>
     <row r="26" spans="1:13">
@@ -1381,37 +1414,37 @@
         <v>14</v>
       </c>
       <c r="B26" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C26" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="D26" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="F26" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="G26" t="s">
-        <v>33</v>
+        <v>37</v>
       </c>
       <c r="H26">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="I26">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="J26">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="K26">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="L26" s="2">
-        <v>46087.82594907407</v>
+        <v>46087.81978009259</v>
       </c>
       <c r="M26" s="2">
-        <v>46087.82975694445</v>
+        <v>46087.81979166667</v>
       </c>
     </row>
     <row r="27" spans="1:13">
@@ -1419,37 +1452,37 @@
         <v>14</v>
       </c>
       <c r="B27" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C27" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="D27" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="F27" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="G27" t="s">
-        <v>33</v>
+        <v>37</v>
       </c>
       <c r="H27">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="I27">
         <v>3</v>
       </c>
       <c r="J27">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="K27">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="L27" s="2">
-        <v>46087.83453703704</v>
+        <v>46087.82594907407</v>
       </c>
       <c r="M27" s="2">
-        <v>46087.83635416667</v>
+        <v>46087.82975694445</v>
       </c>
     </row>
     <row r="28" spans="1:13">
@@ -1457,37 +1490,37 @@
         <v>14</v>
       </c>
       <c r="B28" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C28" t="s">
         <v>23</v>
       </c>
       <c r="D28" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="F28" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="G28" t="s">
-        <v>33</v>
+        <v>37</v>
       </c>
       <c r="H28">
         <v>0</v>
       </c>
       <c r="I28">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="J28">
         <v>0</v>
       </c>
       <c r="K28">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="L28" s="2">
-        <v>46087.83888888889</v>
+        <v>46087.83453703704</v>
       </c>
       <c r="M28" s="2">
-        <v>46087.83888888889</v>
+        <v>46087.83635416667</v>
       </c>
     </row>
     <row r="29" spans="1:13">
@@ -1495,37 +1528,37 @@
         <v>14</v>
       </c>
       <c r="B29" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C29" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="D29" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="F29" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="G29" t="s">
-        <v>33</v>
+        <v>37</v>
       </c>
       <c r="H29">
         <v>0</v>
       </c>
       <c r="I29">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J29">
         <v>0</v>
       </c>
       <c r="K29">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="L29" s="2">
-        <v>46087.84623842593</v>
+        <v>46087.83888888889</v>
       </c>
       <c r="M29" s="2">
-        <v>46087.84766203703</v>
+        <v>46087.83888888889</v>
       </c>
     </row>
     <row r="30" spans="1:13">
@@ -1533,25 +1566,37 @@
         <v>14</v>
       </c>
       <c r="B30" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C30" t="s">
         <v>23</v>
       </c>
       <c r="D30" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="F30" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="G30" t="s">
-        <v>33</v>
+        <v>37</v>
+      </c>
+      <c r="H30">
+        <v>0</v>
+      </c>
+      <c r="I30">
+        <v>2</v>
+      </c>
+      <c r="J30">
+        <v>0</v>
       </c>
       <c r="K30">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="L30" s="2">
-        <v>46088.12640046296</v>
+        <v>46087.84623842593</v>
+      </c>
+      <c r="M30" s="2">
+        <v>46087.84766203703</v>
       </c>
     </row>
     <row r="31" spans="1:13">
@@ -1559,37 +1604,28 @@
         <v>14</v>
       </c>
       <c r="B31" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C31" t="s">
         <v>24</v>
       </c>
       <c r="D31" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="F31" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="G31" t="s">
-        <v>33</v>
-      </c>
-      <c r="H31">
-        <v>0</v>
-      </c>
-      <c r="I31">
-        <v>1</v>
-      </c>
-      <c r="J31">
-        <v>0</v>
+        <v>37</v>
       </c>
       <c r="K31">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="L31" s="2">
-        <v>46088.14489583333</v>
+        <v>46088.12640046296</v>
       </c>
       <c r="M31" s="2">
-        <v>46088.14637731481</v>
+        <v>46103.51736058765</v>
       </c>
     </row>
     <row r="32" spans="1:13">
@@ -1597,25 +1633,37 @@
         <v>14</v>
       </c>
       <c r="B32" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C32" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="D32" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="F32" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="G32" t="s">
-        <v>33</v>
+        <v>37</v>
+      </c>
+      <c r="H32">
+        <v>0</v>
+      </c>
+      <c r="I32">
+        <v>1</v>
+      </c>
+      <c r="J32">
+        <v>0</v>
       </c>
       <c r="K32">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="L32" s="2">
-        <v>46088.1487037037</v>
+        <v>46088.14489583333</v>
+      </c>
+      <c r="M32" s="2">
+        <v>46088.14637731481</v>
       </c>
     </row>
     <row r="33" spans="1:13">
@@ -1623,25 +1671,28 @@
         <v>14</v>
       </c>
       <c r="B33" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C33" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="D33" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="F33" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="G33" t="s">
-        <v>33</v>
+        <v>37</v>
       </c>
       <c r="K33">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="L33" s="2">
-        <v>46088.15003472222</v>
+        <v>46088.1487037037</v>
+      </c>
+      <c r="M33" s="2">
+        <v>46103.51736058765</v>
       </c>
     </row>
     <row r="34" spans="1:13">
@@ -1649,25 +1700,28 @@
         <v>14</v>
       </c>
       <c r="B34" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C34" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="D34" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="F34" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="G34" t="s">
-        <v>33</v>
+        <v>37</v>
       </c>
       <c r="K34">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="L34" s="2">
-        <v>46088.15659722222</v>
+        <v>46088.15003472222</v>
+      </c>
+      <c r="M34" s="2">
+        <v>46103.51736058765</v>
       </c>
     </row>
     <row r="35" spans="1:13">
@@ -1675,25 +1729,28 @@
         <v>14</v>
       </c>
       <c r="B35" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C35" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="D35" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="F35" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="G35" t="s">
-        <v>33</v>
+        <v>37</v>
       </c>
       <c r="K35">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="L35" s="2">
-        <v>46088.16049768519</v>
+        <v>46088.15659722222</v>
+      </c>
+      <c r="M35" s="2">
+        <v>46103.51736058765</v>
       </c>
     </row>
     <row r="36" spans="1:13">
@@ -1701,25 +1758,28 @@
         <v>14</v>
       </c>
       <c r="B36" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C36" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="D36" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="F36" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="G36" t="s">
-        <v>33</v>
+        <v>37</v>
       </c>
       <c r="K36">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="L36" s="2">
-        <v>46088.16061342593</v>
+        <v>46088.16049768519</v>
+      </c>
+      <c r="M36" s="2">
+        <v>46103.51736058765</v>
       </c>
     </row>
     <row r="37" spans="1:13">
@@ -1727,25 +1787,28 @@
         <v>14</v>
       </c>
       <c r="B37" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C37" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="D37" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="F37" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="G37" t="s">
-        <v>33</v>
+        <v>37</v>
       </c>
       <c r="K37">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="L37" s="2">
-        <v>46088.16140046297</v>
+        <v>46088.16061342593</v>
+      </c>
+      <c r="M37" s="2">
+        <v>46103.51736058765</v>
       </c>
     </row>
     <row r="38" spans="1:13">
@@ -1753,25 +1816,28 @@
         <v>14</v>
       </c>
       <c r="B38" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C38" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="D38" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="F38" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="G38" t="s">
-        <v>33</v>
+        <v>37</v>
       </c>
       <c r="K38">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="L38" s="2">
-        <v>46088.16510416667</v>
+        <v>46088.16140046297</v>
+      </c>
+      <c r="M38" s="2">
+        <v>46103.51736058765</v>
       </c>
     </row>
     <row r="39" spans="1:13">
@@ -1779,37 +1845,28 @@
         <v>14</v>
       </c>
       <c r="B39" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C39" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="D39" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="F39" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="G39" t="s">
-        <v>33</v>
-      </c>
-      <c r="H39">
-        <v>0</v>
-      </c>
-      <c r="I39">
-        <v>3</v>
-      </c>
-      <c r="J39">
-        <v>0</v>
+        <v>37</v>
       </c>
       <c r="K39">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="L39" s="2">
-        <v>46088.16806712963</v>
+        <v>46088.16510416667</v>
       </c>
       <c r="M39" s="2">
-        <v>46088.16965277777</v>
+        <v>46103.51736058765</v>
       </c>
     </row>
     <row r="40" spans="1:13">
@@ -1817,25 +1874,37 @@
         <v>14</v>
       </c>
       <c r="B40" t="s">
+        <v>20</v>
+      </c>
+      <c r="C40" t="s">
+        <v>23</v>
+      </c>
+      <c r="D40" t="s">
+        <v>30</v>
+      </c>
+      <c r="F40" t="s">
+        <v>34</v>
+      </c>
+      <c r="G40" t="s">
+        <v>37</v>
+      </c>
+      <c r="H40">
+        <v>0</v>
+      </c>
+      <c r="I40">
+        <v>3</v>
+      </c>
+      <c r="J40">
+        <v>0</v>
+      </c>
+      <c r="K40">
         <v>19</v>
       </c>
-      <c r="C40" t="s">
-        <v>22</v>
-      </c>
-      <c r="D40" t="s">
-        <v>28</v>
-      </c>
-      <c r="F40" t="s">
-        <v>31</v>
-      </c>
-      <c r="G40" t="s">
-        <v>33</v>
-      </c>
-      <c r="K40">
-        <v>21</v>
-      </c>
       <c r="L40" s="2">
-        <v>46088.18351851852</v>
+        <v>46088.16806712963</v>
+      </c>
+      <c r="M40" s="2">
+        <v>46088.16965277777</v>
       </c>
     </row>
     <row r="41" spans="1:13">
@@ -1843,37 +1912,28 @@
         <v>14</v>
       </c>
       <c r="B41" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C41" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="D41" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="F41" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="G41" t="s">
-        <v>33</v>
-      </c>
-      <c r="H41">
-        <v>0</v>
-      </c>
-      <c r="I41">
-        <v>0</v>
-      </c>
-      <c r="J41">
-        <v>0</v>
+        <v>37</v>
       </c>
       <c r="K41">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="L41" s="2">
-        <v>46088.19144675926</v>
+        <v>46088.18351851852</v>
       </c>
       <c r="M41" s="2">
-        <v>46088.19282407407</v>
+        <v>46103.51736058765</v>
       </c>
     </row>
     <row r="42" spans="1:13">
@@ -1881,37 +1941,37 @@
         <v>14</v>
       </c>
       <c r="B42" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C42" t="s">
+        <v>23</v>
+      </c>
+      <c r="D42" t="s">
+        <v>30</v>
+      </c>
+      <c r="F42" t="s">
+        <v>34</v>
+      </c>
+      <c r="G42" t="s">
+        <v>37</v>
+      </c>
+      <c r="H42">
+        <v>0</v>
+      </c>
+      <c r="I42">
+        <v>0</v>
+      </c>
+      <c r="J42">
+        <v>0</v>
+      </c>
+      <c r="K42">
         <v>22</v>
       </c>
-      <c r="D42" t="s">
-        <v>28</v>
-      </c>
-      <c r="F42" t="s">
-        <v>31</v>
-      </c>
-      <c r="G42" t="s">
-        <v>33</v>
-      </c>
-      <c r="H42">
-        <v>0</v>
-      </c>
-      <c r="I42">
-        <v>0</v>
-      </c>
-      <c r="J42">
-        <v>0</v>
-      </c>
-      <c r="K42">
-        <v>24</v>
-      </c>
       <c r="L42" s="2">
-        <v>46088.19351851852</v>
+        <v>46088.19144675926</v>
       </c>
       <c r="M42" s="2">
-        <v>46088.19489583333</v>
+        <v>46088.19282407407</v>
       </c>
     </row>
     <row r="43" spans="1:13">
@@ -1919,25 +1979,37 @@
         <v>14</v>
       </c>
       <c r="B43" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C43" t="s">
         <v>23</v>
       </c>
       <c r="D43" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="F43" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="G43" t="s">
-        <v>33</v>
+        <v>37</v>
+      </c>
+      <c r="H43">
+        <v>0</v>
+      </c>
+      <c r="I43">
+        <v>0</v>
+      </c>
+      <c r="J43">
+        <v>0</v>
       </c>
       <c r="K43">
-        <v>2</v>
+        <v>24</v>
       </c>
       <c r="L43" s="2">
-        <v>46087.81545138889</v>
+        <v>46088.19351851852</v>
+      </c>
+      <c r="M43" s="2">
+        <v>46088.19489583333</v>
       </c>
     </row>
     <row r="44" spans="1:13">
@@ -1945,37 +2017,28 @@
         <v>14</v>
       </c>
       <c r="B44" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C44" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="D44" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="F44" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="G44" t="s">
-        <v>33</v>
-      </c>
-      <c r="H44">
-        <v>0</v>
-      </c>
-      <c r="I44">
-        <v>1</v>
-      </c>
-      <c r="J44">
-        <v>0</v>
+        <v>37</v>
       </c>
       <c r="K44">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="L44" s="2">
-        <v>46087.82997685186</v>
+        <v>46087.81545138889</v>
       </c>
       <c r="M44" s="2">
-        <v>46087.8316550926</v>
+        <v>46103.51736057608</v>
       </c>
     </row>
     <row r="45" spans="1:13">
@@ -1983,25 +2046,37 @@
         <v>14</v>
       </c>
       <c r="B45" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C45" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="D45" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="F45" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="G45" t="s">
-        <v>33</v>
+        <v>37</v>
+      </c>
+      <c r="H45">
+        <v>0</v>
+      </c>
+      <c r="I45">
+        <v>1</v>
+      </c>
+      <c r="J45">
+        <v>0</v>
       </c>
       <c r="K45">
-        <v>20</v>
+        <v>6</v>
       </c>
       <c r="L45" s="2">
-        <v>46088.17351851852</v>
+        <v>46087.82997685186</v>
+      </c>
+      <c r="M45" s="2">
+        <v>46087.8316550926</v>
       </c>
     </row>
     <row r="46" spans="1:13">
@@ -2009,37 +2084,28 @@
         <v>14</v>
       </c>
       <c r="B46" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C46" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D46" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="F46" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="G46" t="s">
-        <v>33</v>
-      </c>
-      <c r="H46">
-        <v>0</v>
-      </c>
-      <c r="I46">
-        <v>7</v>
-      </c>
-      <c r="J46">
-        <v>0</v>
+        <v>37</v>
       </c>
       <c r="K46">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="L46" s="2">
-        <v>46088.19304398148</v>
+        <v>46088.17351851852</v>
       </c>
       <c r="M46" s="2">
-        <v>46088.19311342593</v>
+        <v>46103.51736058765</v>
       </c>
     </row>
     <row r="47" spans="1:13">
@@ -2047,37 +2113,37 @@
         <v>14</v>
       </c>
       <c r="B47" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C47" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="D47" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="F47" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="G47" t="s">
-        <v>33</v>
+        <v>37</v>
       </c>
       <c r="H47">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="I47">
         <v>7</v>
       </c>
       <c r="J47">
-        <v>42.85714285714285</v>
+        <v>0</v>
       </c>
       <c r="K47">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="L47" s="2">
-        <v>46088.75755787037</v>
+        <v>46088.19304398148</v>
       </c>
       <c r="M47" s="2">
-        <v>46088.75893518519</v>
+        <v>46088.19311342593</v>
       </c>
     </row>
     <row r="48" spans="1:13">
@@ -2085,37 +2151,37 @@
         <v>14</v>
       </c>
       <c r="B48" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C48" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D48" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="F48" t="s">
-        <v>30</v>
+        <v>35</v>
       </c>
       <c r="G48" t="s">
-        <v>33</v>
+        <v>37</v>
       </c>
       <c r="H48">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="I48">
         <v>7</v>
       </c>
       <c r="J48">
-        <v>57.14285714285714</v>
+        <v>42.85714285714285</v>
       </c>
       <c r="K48">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="L48" s="2">
-        <v>46088.77844907407</v>
+        <v>46088.75755787037</v>
       </c>
       <c r="M48" s="2">
-        <v>46088.77982638889</v>
+        <v>46088.75893518519</v>
       </c>
     </row>
     <row r="49" spans="1:13">
@@ -2123,37 +2189,37 @@
         <v>14</v>
       </c>
       <c r="B49" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C49" t="s">
+        <v>25</v>
+      </c>
+      <c r="D49" t="s">
+        <v>30</v>
+      </c>
+      <c r="F49" t="s">
+        <v>33</v>
+      </c>
+      <c r="G49" t="s">
+        <v>37</v>
+      </c>
+      <c r="H49">
+        <v>4</v>
+      </c>
+      <c r="I49">
+        <v>7</v>
+      </c>
+      <c r="J49">
+        <v>57.14285714285714</v>
+      </c>
+      <c r="K49">
         <v>26</v>
       </c>
-      <c r="D49" t="s">
-        <v>29</v>
-      </c>
-      <c r="F49" t="s">
-        <v>26</v>
-      </c>
-      <c r="G49" t="s">
-        <v>26</v>
-      </c>
-      <c r="H49">
-        <v>0</v>
-      </c>
-      <c r="I49">
-        <v>3</v>
-      </c>
-      <c r="J49">
-        <v>0</v>
-      </c>
-      <c r="K49">
-        <v>1</v>
-      </c>
       <c r="L49" s="2">
-        <v>46087.82002314815</v>
+        <v>46088.77844907407</v>
       </c>
       <c r="M49" s="2">
-        <v>46087.82015046296</v>
+        <v>46088.77982638889</v>
       </c>
     </row>
     <row r="50" spans="1:13">
@@ -2164,22 +2230,22 @@
         <v>20</v>
       </c>
       <c r="C50" t="s">
-        <v>22</v>
+        <v>28</v>
       </c>
       <c r="D50" t="s">
+        <v>31</v>
+      </c>
+      <c r="F50" t="s">
         <v>28</v>
       </c>
-      <c r="F50" t="s">
-        <v>31</v>
-      </c>
       <c r="G50" t="s">
-        <v>33</v>
+        <v>28</v>
       </c>
       <c r="H50">
         <v>0</v>
       </c>
       <c r="I50">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="J50">
         <v>0</v>
@@ -2188,10 +2254,10 @@
         <v>1</v>
       </c>
       <c r="L50" s="2">
-        <v>46087.61813657408</v>
+        <v>46087.82002314815</v>
       </c>
       <c r="M50" s="2">
-        <v>46087.61813657408</v>
+        <v>46087.82015046296</v>
       </c>
     </row>
     <row r="51" spans="1:13">
@@ -2199,37 +2265,37 @@
         <v>14</v>
       </c>
       <c r="B51" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C51" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="D51" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="F51" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="G51" t="s">
-        <v>33</v>
+        <v>37</v>
       </c>
       <c r="H51">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="I51">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="J51">
-        <v>85.71428571428571</v>
+        <v>0</v>
       </c>
       <c r="K51">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L51" s="2">
-        <v>46087.61918981482</v>
+        <v>46087.61813657408</v>
       </c>
       <c r="M51" s="2">
-        <v>46087.61979166666</v>
+        <v>46087.61813657408</v>
       </c>
     </row>
     <row r="52" spans="1:13">
@@ -2237,37 +2303,37 @@
         <v>14</v>
       </c>
       <c r="B52" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C52" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="D52" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="F52" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="G52" t="s">
-        <v>33</v>
+        <v>37</v>
       </c>
       <c r="H52">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="I52">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="J52">
-        <v>0</v>
+        <v>85.71428571428571</v>
       </c>
       <c r="K52">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="L52" s="2">
-        <v>46087.75652777778</v>
+        <v>46087.61918981482</v>
       </c>
       <c r="M52" s="2">
-        <v>46087.77236111111</v>
+        <v>46087.61979166666</v>
       </c>
     </row>
     <row r="53" spans="1:13">
@@ -2275,37 +2341,37 @@
         <v>14</v>
       </c>
       <c r="B53" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C53" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="D53" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="F53" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="G53" t="s">
-        <v>33</v>
+        <v>37</v>
       </c>
       <c r="H53">
         <v>0</v>
       </c>
       <c r="I53">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="J53">
         <v>0</v>
       </c>
       <c r="K53">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="L53" s="2">
-        <v>46087.72322916667</v>
+        <v>46087.75652777778</v>
       </c>
       <c r="M53" s="2">
-        <v>46087.72322916667</v>
+        <v>46087.77236111111</v>
       </c>
     </row>
     <row r="54" spans="1:13">
@@ -2313,19 +2379,19 @@
         <v>14</v>
       </c>
       <c r="B54" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C54" t="s">
         <v>23</v>
       </c>
       <c r="D54" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="F54" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="G54" t="s">
-        <v>33</v>
+        <v>37</v>
       </c>
       <c r="H54">
         <v>0</v>
@@ -2337,13 +2403,13 @@
         <v>0</v>
       </c>
       <c r="K54">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="L54" s="2">
-        <v>46087.72596064815</v>
+        <v>46087.72322916667</v>
       </c>
       <c r="M54" s="2">
-        <v>46087.72596064815</v>
+        <v>46087.72322916667</v>
       </c>
     </row>
     <row r="55" spans="1:13">
@@ -2351,37 +2417,37 @@
         <v>14</v>
       </c>
       <c r="B55" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C55" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="D55" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="F55" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="G55" t="s">
-        <v>33</v>
+        <v>37</v>
       </c>
       <c r="H55">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="I55">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="J55">
-        <v>85.71428571428571</v>
+        <v>0</v>
       </c>
       <c r="K55">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="L55" s="2">
-        <v>46087.78849537037</v>
+        <v>46087.72596064815</v>
       </c>
       <c r="M55" s="2">
-        <v>46087.80008101852</v>
+        <v>46087.72596064815</v>
       </c>
     </row>
     <row r="56" spans="1:13">
@@ -2389,36 +2455,74 @@
         <v>14</v>
       </c>
       <c r="B56" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C56" t="s">
         <v>24</v>
       </c>
       <c r="D56" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="F56" t="s">
-        <v>30</v>
+        <v>35</v>
       </c>
       <c r="G56" t="s">
+        <v>37</v>
+      </c>
+      <c r="H56">
+        <v>6</v>
+      </c>
+      <c r="I56">
+        <v>7</v>
+      </c>
+      <c r="J56">
+        <v>85.71428571428571</v>
+      </c>
+      <c r="K56">
+        <v>7</v>
+      </c>
+      <c r="L56" s="2">
+        <v>46087.78849537037</v>
+      </c>
+      <c r="M56" s="2">
+        <v>46087.80008101852</v>
+      </c>
+    </row>
+    <row r="57" spans="1:13">
+      <c r="A57" t="s">
+        <v>14</v>
+      </c>
+      <c r="B57" t="s">
+        <v>21</v>
+      </c>
+      <c r="C57" t="s">
+        <v>25</v>
+      </c>
+      <c r="D57" t="s">
+        <v>30</v>
+      </c>
+      <c r="F57" t="s">
         <v>33</v>
       </c>
-      <c r="H56">
-        <v>0</v>
-      </c>
-      <c r="I56">
-        <v>0</v>
-      </c>
-      <c r="J56">
-        <v>0</v>
-      </c>
-      <c r="K56">
+      <c r="G57" t="s">
+        <v>37</v>
+      </c>
+      <c r="H57">
+        <v>0</v>
+      </c>
+      <c r="I57">
+        <v>0</v>
+      </c>
+      <c r="J57">
+        <v>0</v>
+      </c>
+      <c r="K57">
         <v>3</v>
       </c>
-      <c r="L56" s="2">
+      <c r="L57" s="2">
         <v>46087.71842592592</v>
       </c>
-      <c r="M56" s="2">
+      <c r="M57" s="2">
         <v>46087.71842592592</v>
       </c>
     </row>

</xml_diff>